<commit_message>
Make pivot table layout Excel-compliant (row/column items)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MkborAFWdPjADAzhkntAHn
</commit_message>
<xml_diff>
--- a/품목별_원가비교_대시보드.xlsx
+++ b/품목별_원가비교_대시보드.xlsx
@@ -10410,9 +10410,103 @@
     <field x="2"/>
     <field x="3"/>
   </rowFields>
+  <rowItems count="25">
+    <i>
+      <x/>
+      <x/>
+      <x/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i r="2">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="3"/>
+    </i>
+    <i r="2">
+      <x v="4"/>
+    </i>
+    <i r="2">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+      <x/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i r="2">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="3"/>
+    </i>
+    <i r="2">
+      <x v="4"/>
+    </i>
+    <i r="2">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="1"/>
+      <x/>
+      <x/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i r="2">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="3"/>
+    </i>
+    <i r="2">
+      <x v="4"/>
+    </i>
+    <i r="2">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+      <x/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i r="2">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="3"/>
+    </i>
+    <i r="2">
+      <x v="4"/>
+    </i>
+    <i r="2">
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
   <colFields count="1">
     <field x="-2"/>
   </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+  </colItems>
   <pageFields count="1">
     <pageField fld="0" hier="-1"/>
   </pageFields>

</xml_diff>